<commit_message>
fix: tune generator re-sit bonus for a realistic pass-rate trend
</commit_message>
<xml_diff>
--- a/data/sample/results_2023_dec.xlsx
+++ b/data/sample/results_2023_dec.xlsx
@@ -521,10 +521,12 @@
           <t>2023-Dec</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr"/>
+      <c r="I2" t="n">
+        <v>64</v>
+      </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Absent</t>
+          <t>Sat</t>
         </is>
       </c>
     </row>
@@ -570,7 +572,7 @@
         </is>
       </c>
       <c r="I3" t="n">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
@@ -620,7 +622,7 @@
         </is>
       </c>
       <c r="I4" t="n">
-        <v>61</v>
+        <v>72</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
@@ -670,7 +672,7 @@
         </is>
       </c>
       <c r="I5" t="n">
-        <v>62</v>
+        <v>54</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
@@ -720,7 +722,7 @@
         </is>
       </c>
       <c r="I6" t="n">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
@@ -770,7 +772,7 @@
         </is>
       </c>
       <c r="I7" t="n">
-        <v>75</v>
+        <v>60</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
@@ -870,7 +872,7 @@
         </is>
       </c>
       <c r="I9" t="n">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="J9" t="inlineStr">
         <is>
@@ -920,7 +922,7 @@
         </is>
       </c>
       <c r="I10" t="n">
-        <v>69</v>
+        <v>56</v>
       </c>
       <c r="J10" t="inlineStr">
         <is>
@@ -970,7 +972,7 @@
         </is>
       </c>
       <c r="I11" t="n">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="J11" t="inlineStr">
         <is>
@@ -1019,12 +1021,10 @@
           <t>2023-Dec</t>
         </is>
       </c>
-      <c r="I12" t="n">
-        <v>74</v>
-      </c>
+      <c r="I12" t="inlineStr"/>
       <c r="J12" t="inlineStr">
         <is>
-          <t>Sat</t>
+          <t>Absent</t>
         </is>
       </c>
     </row>
@@ -1070,7 +1070,7 @@
         </is>
       </c>
       <c r="I13" t="n">
-        <v>59</v>
+        <v>75</v>
       </c>
       <c r="J13" t="inlineStr">
         <is>
@@ -1120,7 +1120,7 @@
         </is>
       </c>
       <c r="I14" t="n">
-        <v>71</v>
+        <v>64</v>
       </c>
       <c r="J14" t="inlineStr">
         <is>
@@ -1170,7 +1170,7 @@
         </is>
       </c>
       <c r="I15" t="n">
-        <v>70</v>
+        <v>62</v>
       </c>
       <c r="J15" t="inlineStr">
         <is>
@@ -1269,12 +1269,10 @@
           <t>2023-Dec</t>
         </is>
       </c>
-      <c r="I17" t="n">
-        <v>50</v>
-      </c>
+      <c r="I17" t="inlineStr"/>
       <c r="J17" t="inlineStr">
         <is>
-          <t>Sat</t>
+          <t>Absent</t>
         </is>
       </c>
     </row>
@@ -1320,7 +1318,7 @@
         </is>
       </c>
       <c r="I18" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="J18" t="inlineStr">
         <is>
@@ -1370,7 +1368,7 @@
         </is>
       </c>
       <c r="I19" t="n">
-        <v>43</v>
+        <v>55</v>
       </c>
       <c r="J19" t="inlineStr">
         <is>
@@ -1420,7 +1418,7 @@
         </is>
       </c>
       <c r="I20" t="n">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="J20" t="inlineStr">
         <is>
@@ -1470,7 +1468,7 @@
         </is>
       </c>
       <c r="I21" t="n">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="J21" t="inlineStr">
         <is>
@@ -1520,7 +1518,7 @@
         </is>
       </c>
       <c r="I22" t="n">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="J22" t="inlineStr">
         <is>
@@ -1570,7 +1568,7 @@
         </is>
       </c>
       <c r="I23" t="n">
-        <v>59</v>
+        <v>50</v>
       </c>
       <c r="J23" t="inlineStr">
         <is>
@@ -1620,7 +1618,7 @@
         </is>
       </c>
       <c r="I24" t="n">
-        <v>63</v>
+        <v>45</v>
       </c>
       <c r="J24" t="inlineStr">
         <is>
@@ -1670,7 +1668,7 @@
         </is>
       </c>
       <c r="I25" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="J25" t="inlineStr">
         <is>
@@ -1720,7 +1718,7 @@
         </is>
       </c>
       <c r="I26" t="n">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="J26" t="inlineStr">
         <is>
@@ -1770,7 +1768,7 @@
         </is>
       </c>
       <c r="I27" t="n">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="J27" t="inlineStr">
         <is>
@@ -1820,7 +1818,7 @@
         </is>
       </c>
       <c r="I28" t="n">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="J28" t="inlineStr">
         <is>
@@ -1870,7 +1868,7 @@
         </is>
       </c>
       <c r="I29" t="n">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="J29" t="inlineStr">
         <is>
@@ -1920,7 +1918,7 @@
         </is>
       </c>
       <c r="I30" t="n">
-        <v>77</v>
+        <v>69</v>
       </c>
       <c r="J30" t="inlineStr">
         <is>
@@ -1970,7 +1968,7 @@
         </is>
       </c>
       <c r="I31" t="n">
-        <v>69</v>
+        <v>60</v>
       </c>
       <c r="J31" t="inlineStr">
         <is>
@@ -2020,7 +2018,7 @@
         </is>
       </c>
       <c r="I32" t="n">
-        <v>77</v>
+        <v>62</v>
       </c>
       <c r="J32" t="inlineStr">
         <is>
@@ -2070,7 +2068,7 @@
         </is>
       </c>
       <c r="I33" t="n">
-        <v>69</v>
+        <v>50</v>
       </c>
       <c r="J33" t="inlineStr">
         <is>
@@ -2120,7 +2118,7 @@
         </is>
       </c>
       <c r="I34" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="J34" t="inlineStr">
         <is>
@@ -2170,7 +2168,7 @@
         </is>
       </c>
       <c r="I35" t="n">
-        <v>53</v>
+        <v>65</v>
       </c>
       <c r="J35" t="inlineStr">
         <is>
@@ -2220,7 +2218,7 @@
         </is>
       </c>
       <c r="I36" t="n">
-        <v>63</v>
+        <v>78</v>
       </c>
       <c r="J36" t="inlineStr">
         <is>
@@ -2270,7 +2268,7 @@
         </is>
       </c>
       <c r="I37" t="n">
-        <v>67</v>
+        <v>75</v>
       </c>
       <c r="J37" t="inlineStr">
         <is>
@@ -2320,7 +2318,7 @@
         </is>
       </c>
       <c r="I38" t="n">
-        <v>75</v>
+        <v>57</v>
       </c>
       <c r="J38" t="inlineStr">
         <is>
@@ -2370,7 +2368,7 @@
         </is>
       </c>
       <c r="I39" t="n">
-        <v>57</v>
+        <v>78</v>
       </c>
       <c r="J39" t="inlineStr">
         <is>
@@ -2420,7 +2418,7 @@
         </is>
       </c>
       <c r="I40" t="n">
-        <v>75</v>
+        <v>64</v>
       </c>
       <c r="J40" t="inlineStr">
         <is>
@@ -2470,7 +2468,7 @@
         </is>
       </c>
       <c r="I41" t="n">
-        <v>66</v>
+        <v>76</v>
       </c>
       <c r="J41" t="inlineStr">
         <is>
@@ -2520,7 +2518,7 @@
         </is>
       </c>
       <c r="I42" t="n">
-        <v>69</v>
+        <v>82</v>
       </c>
       <c r="J42" t="inlineStr">
         <is>
@@ -2570,7 +2568,7 @@
         </is>
       </c>
       <c r="I43" t="n">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="J43" t="inlineStr">
         <is>
@@ -2620,7 +2618,7 @@
         </is>
       </c>
       <c r="I44" t="n">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="J44" t="inlineStr">
         <is>
@@ -2670,7 +2668,7 @@
         </is>
       </c>
       <c r="I45" t="n">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="J45" t="inlineStr">
         <is>
@@ -2720,7 +2718,7 @@
         </is>
       </c>
       <c r="I46" t="n">
-        <v>43</v>
+        <v>50</v>
       </c>
       <c r="J46" t="inlineStr">
         <is>
@@ -2770,7 +2768,7 @@
         </is>
       </c>
       <c r="I47" t="n">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="J47" t="inlineStr">
         <is>
@@ -2820,7 +2818,7 @@
         </is>
       </c>
       <c r="I48" t="n">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="J48" t="inlineStr">
         <is>
@@ -2870,7 +2868,7 @@
         </is>
       </c>
       <c r="I49" t="n">
-        <v>56</v>
+        <v>49</v>
       </c>
       <c r="J49" t="inlineStr">
         <is>
@@ -2920,7 +2918,7 @@
         </is>
       </c>
       <c r="I50" t="n">
-        <v>43</v>
+        <v>57</v>
       </c>
       <c r="J50" t="inlineStr">
         <is>
@@ -2970,7 +2968,7 @@
         </is>
       </c>
       <c r="I51" t="n">
-        <v>49</v>
+        <v>37</v>
       </c>
       <c r="J51" t="inlineStr">
         <is>
@@ -3020,7 +3018,7 @@
         </is>
       </c>
       <c r="I52" t="n">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="J52" t="inlineStr">
         <is>
@@ -3070,7 +3068,7 @@
         </is>
       </c>
       <c r="I53" t="n">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="J53" t="inlineStr">
         <is>
@@ -3120,7 +3118,7 @@
         </is>
       </c>
       <c r="I54" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="J54" t="inlineStr">
         <is>
@@ -3170,7 +3168,7 @@
         </is>
       </c>
       <c r="I55" t="n">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="J55" t="inlineStr">
         <is>
@@ -3220,7 +3218,7 @@
         </is>
       </c>
       <c r="I56" t="n">
-        <v>59</v>
+        <v>68</v>
       </c>
       <c r="J56" t="inlineStr">
         <is>
@@ -3270,7 +3268,7 @@
         </is>
       </c>
       <c r="I57" t="n">
-        <v>66</v>
+        <v>51</v>
       </c>
       <c r="J57" t="inlineStr">
         <is>
@@ -3320,7 +3318,7 @@
         </is>
       </c>
       <c r="I58" t="n">
-        <v>65</v>
+        <v>74</v>
       </c>
       <c r="J58" t="inlineStr">
         <is>
@@ -3370,7 +3368,7 @@
         </is>
       </c>
       <c r="I59" t="n">
-        <v>67</v>
+        <v>75</v>
       </c>
       <c r="J59" t="inlineStr">
         <is>
@@ -3420,7 +3418,7 @@
         </is>
       </c>
       <c r="I60" t="n">
-        <v>45</v>
+        <v>62</v>
       </c>
       <c r="J60" t="inlineStr">
         <is>
@@ -3470,7 +3468,7 @@
         </is>
       </c>
       <c r="I61" t="n">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="J61" t="inlineStr">
         <is>
@@ -3520,7 +3518,7 @@
         </is>
       </c>
       <c r="I62" t="n">
-        <v>65</v>
+        <v>83</v>
       </c>
       <c r="J62" t="inlineStr">
         <is>
@@ -3570,7 +3568,7 @@
         </is>
       </c>
       <c r="I63" t="n">
-        <v>86</v>
+        <v>76</v>
       </c>
       <c r="J63" t="inlineStr">
         <is>
@@ -3620,7 +3618,7 @@
         </is>
       </c>
       <c r="I64" t="n">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="J64" t="inlineStr">
         <is>
@@ -3669,10 +3667,12 @@
           <t>2023-Dec</t>
         </is>
       </c>
-      <c r="I65" t="inlineStr"/>
+      <c r="I65" t="n">
+        <v>56</v>
+      </c>
       <c r="J65" t="inlineStr">
         <is>
-          <t>Absent</t>
+          <t>Sat</t>
         </is>
       </c>
     </row>
@@ -3718,7 +3718,7 @@
         </is>
       </c>
       <c r="I66" t="n">
-        <v>68</v>
+        <v>77</v>
       </c>
       <c r="J66" t="inlineStr">
         <is>
@@ -3768,7 +3768,7 @@
         </is>
       </c>
       <c r="I67" t="n">
-        <v>54</v>
+        <v>63</v>
       </c>
       <c r="J67" t="inlineStr">
         <is>
@@ -3818,7 +3818,7 @@
         </is>
       </c>
       <c r="I68" t="n">
-        <v>77</v>
+        <v>57</v>
       </c>
       <c r="J68" t="inlineStr">
         <is>
@@ -3868,7 +3868,7 @@
         </is>
       </c>
       <c r="I69" t="n">
-        <v>62</v>
+        <v>73</v>
       </c>
       <c r="J69" t="inlineStr">
         <is>
@@ -3918,7 +3918,7 @@
         </is>
       </c>
       <c r="I70" t="n">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="J70" t="inlineStr">
         <is>
@@ -3968,7 +3968,7 @@
         </is>
       </c>
       <c r="I71" t="n">
-        <v>52</v>
+        <v>42</v>
       </c>
       <c r="J71" t="inlineStr">
         <is>
@@ -4017,10 +4017,12 @@
           <t>2023-Dec</t>
         </is>
       </c>
-      <c r="I72" t="inlineStr"/>
+      <c r="I72" t="n">
+        <v>80</v>
+      </c>
       <c r="J72" t="inlineStr">
         <is>
-          <t>Absent</t>
+          <t>Sat</t>
         </is>
       </c>
     </row>
@@ -4066,7 +4068,7 @@
         </is>
       </c>
       <c r="I73" t="n">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="J73" t="inlineStr">
         <is>
@@ -4116,7 +4118,7 @@
         </is>
       </c>
       <c r="I74" t="n">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="J74" t="inlineStr">
         <is>
@@ -4166,7 +4168,7 @@
         </is>
       </c>
       <c r="I75" t="n">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="J75" t="inlineStr">
         <is>
@@ -4216,7 +4218,7 @@
         </is>
       </c>
       <c r="I76" t="n">
-        <v>65</v>
+        <v>55</v>
       </c>
       <c r="J76" t="inlineStr">
         <is>
@@ -4266,7 +4268,7 @@
         </is>
       </c>
       <c r="I77" t="n">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="J77" t="inlineStr">
         <is>
@@ -4316,7 +4318,7 @@
         </is>
       </c>
       <c r="I78" t="n">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="J78" t="inlineStr">
         <is>
@@ -4366,7 +4368,7 @@
         </is>
       </c>
       <c r="I79" t="n">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="J79" t="inlineStr">
         <is>
@@ -4416,7 +4418,7 @@
         </is>
       </c>
       <c r="I80" t="n">
-        <v>58</v>
+        <v>71</v>
       </c>
       <c r="J80" t="inlineStr">
         <is>
@@ -4466,7 +4468,7 @@
         </is>
       </c>
       <c r="I81" t="n">
-        <v>60</v>
+        <v>53</v>
       </c>
       <c r="J81" t="inlineStr">
         <is>
@@ -4516,7 +4518,7 @@
         </is>
       </c>
       <c r="I82" t="n">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="J82" t="inlineStr">
         <is>
@@ -4566,7 +4568,7 @@
         </is>
       </c>
       <c r="I83" t="n">
-        <v>70</v>
+        <v>63</v>
       </c>
       <c r="J83" t="inlineStr">
         <is>
@@ -4616,7 +4618,7 @@
         </is>
       </c>
       <c r="I84" t="n">
-        <v>63</v>
+        <v>74</v>
       </c>
       <c r="J84" t="inlineStr">
         <is>
@@ -4666,7 +4668,7 @@
         </is>
       </c>
       <c r="I85" t="n">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="J85" t="inlineStr">
         <is>
@@ -4716,7 +4718,7 @@
         </is>
       </c>
       <c r="I86" t="n">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="J86" t="inlineStr">
         <is>
@@ -4766,7 +4768,7 @@
         </is>
       </c>
       <c r="I87" t="n">
-        <v>72</v>
+        <v>57</v>
       </c>
       <c r="J87" t="inlineStr">
         <is>
@@ -4866,7 +4868,7 @@
         </is>
       </c>
       <c r="I89" t="n">
-        <v>66</v>
+        <v>53</v>
       </c>
       <c r="J89" t="inlineStr">
         <is>
@@ -4916,7 +4918,7 @@
         </is>
       </c>
       <c r="I90" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="J90" t="inlineStr">
         <is>
@@ -4965,10 +4967,12 @@
           <t>2023-Dec</t>
         </is>
       </c>
-      <c r="I91" t="inlineStr"/>
+      <c r="I91" t="n">
+        <v>45</v>
+      </c>
       <c r="J91" t="inlineStr">
         <is>
-          <t>Absent</t>
+          <t>Sat</t>
         </is>
       </c>
     </row>
@@ -5014,7 +5018,7 @@
         </is>
       </c>
       <c r="I92" t="n">
-        <v>50</v>
+        <v>61</v>
       </c>
       <c r="J92" t="inlineStr">
         <is>
@@ -5064,7 +5068,7 @@
         </is>
       </c>
       <c r="I93" t="n">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="J93" t="inlineStr">
         <is>
@@ -5114,7 +5118,7 @@
         </is>
       </c>
       <c r="I94" t="n">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="J94" t="inlineStr">
         <is>
@@ -5164,7 +5168,7 @@
         </is>
       </c>
       <c r="I95" t="n">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="J95" t="inlineStr">
         <is>
@@ -5214,7 +5218,7 @@
         </is>
       </c>
       <c r="I96" t="n">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="J96" t="inlineStr">
         <is>
@@ -5264,7 +5268,7 @@
         </is>
       </c>
       <c r="I97" t="n">
-        <v>72</v>
+        <v>60</v>
       </c>
       <c r="J97" t="inlineStr">
         <is>
@@ -5314,7 +5318,7 @@
         </is>
       </c>
       <c r="I98" t="n">
-        <v>38</v>
+        <v>55</v>
       </c>
       <c r="J98" t="inlineStr">
         <is>
@@ -5364,7 +5368,7 @@
         </is>
       </c>
       <c r="I99" t="n">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="J99" t="inlineStr">
         <is>
@@ -5414,7 +5418,7 @@
         </is>
       </c>
       <c r="I100" t="n">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="J100" t="inlineStr">
         <is>
@@ -5464,7 +5468,7 @@
         </is>
       </c>
       <c r="I101" t="n">
-        <v>56</v>
+        <v>66</v>
       </c>
       <c r="J101" t="inlineStr">
         <is>
@@ -5514,7 +5518,7 @@
         </is>
       </c>
       <c r="I102" t="n">
-        <v>82</v>
+        <v>53</v>
       </c>
       <c r="J102" t="inlineStr">
         <is>
@@ -5564,7 +5568,7 @@
         </is>
       </c>
       <c r="I103" t="n">
-        <v>66</v>
+        <v>76</v>
       </c>
       <c r="J103" t="inlineStr">
         <is>
@@ -5613,10 +5617,12 @@
           <t>2023-Dec</t>
         </is>
       </c>
-      <c r="I104" t="inlineStr"/>
+      <c r="I104" t="n">
+        <v>95</v>
+      </c>
       <c r="J104" t="inlineStr">
         <is>
-          <t>Absent</t>
+          <t>Sat</t>
         </is>
       </c>
     </row>
@@ -5662,7 +5668,7 @@
         </is>
       </c>
       <c r="I105" t="n">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="J105" t="inlineStr">
         <is>
@@ -5712,7 +5718,7 @@
         </is>
       </c>
       <c r="I106" t="n">
-        <v>55</v>
+        <v>78</v>
       </c>
       <c r="J106" t="inlineStr">
         <is>
@@ -5761,12 +5767,10 @@
           <t>2023-Dec</t>
         </is>
       </c>
-      <c r="I107" t="n">
-        <v>62</v>
-      </c>
+      <c r="I107" t="inlineStr"/>
       <c r="J107" t="inlineStr">
         <is>
-          <t>Sat</t>
+          <t>Absent</t>
         </is>
       </c>
     </row>
@@ -5811,12 +5815,10 @@
           <t>2023-Dec</t>
         </is>
       </c>
-      <c r="I108" t="n">
-        <v>62</v>
-      </c>
+      <c r="I108" t="inlineStr"/>
       <c r="J108" t="inlineStr">
         <is>
-          <t>Sat</t>
+          <t>Absent</t>
         </is>
       </c>
     </row>
@@ -5862,7 +5864,7 @@
         </is>
       </c>
       <c r="I109" t="n">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="J109" t="inlineStr">
         <is>
@@ -5912,7 +5914,7 @@
         </is>
       </c>
       <c r="I110" t="n">
-        <v>63</v>
+        <v>73</v>
       </c>
       <c r="J110" t="inlineStr">
         <is>
@@ -5962,7 +5964,7 @@
         </is>
       </c>
       <c r="I111" t="n">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="J111" t="inlineStr">
         <is>
@@ -6012,7 +6014,7 @@
         </is>
       </c>
       <c r="I112" t="n">
-        <v>75</v>
+        <v>63</v>
       </c>
       <c r="J112" t="inlineStr">
         <is>
@@ -6061,10 +6063,12 @@
           <t>2023-Dec</t>
         </is>
       </c>
-      <c r="I113" t="inlineStr"/>
+      <c r="I113" t="n">
+        <v>67</v>
+      </c>
       <c r="J113" t="inlineStr">
         <is>
-          <t>Absent</t>
+          <t>Sat</t>
         </is>
       </c>
     </row>
@@ -6109,12 +6113,10 @@
           <t>2023-Dec</t>
         </is>
       </c>
-      <c r="I114" t="n">
-        <v>65</v>
-      </c>
+      <c r="I114" t="inlineStr"/>
       <c r="J114" t="inlineStr">
         <is>
-          <t>Sat</t>
+          <t>Absent</t>
         </is>
       </c>
     </row>
@@ -6160,7 +6162,7 @@
         </is>
       </c>
       <c r="I115" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="J115" t="inlineStr">
         <is>
@@ -6210,7 +6212,7 @@
         </is>
       </c>
       <c r="I116" t="n">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="J116" t="inlineStr">
         <is>
@@ -6260,7 +6262,7 @@
         </is>
       </c>
       <c r="I117" t="n">
-        <v>54</v>
+        <v>63</v>
       </c>
       <c r="J117" t="inlineStr">
         <is>
@@ -6310,7 +6312,7 @@
         </is>
       </c>
       <c r="I118" t="n">
-        <v>73</v>
+        <v>60</v>
       </c>
       <c r="J118" t="inlineStr">
         <is>
@@ -6360,7 +6362,7 @@
         </is>
       </c>
       <c r="I119" t="n">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="J119" t="inlineStr">
         <is>
@@ -6409,12 +6411,10 @@
           <t>2023-Dec</t>
         </is>
       </c>
-      <c r="I120" t="n">
-        <v>44</v>
-      </c>
+      <c r="I120" t="inlineStr"/>
       <c r="J120" t="inlineStr">
         <is>
-          <t>Sat</t>
+          <t>Absent</t>
         </is>
       </c>
     </row>
@@ -6460,7 +6460,7 @@
         </is>
       </c>
       <c r="I121" t="n">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="J121" t="inlineStr">
         <is>
@@ -6510,7 +6510,7 @@
         </is>
       </c>
       <c r="I122" t="n">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="J122" t="inlineStr">
         <is>
@@ -6560,7 +6560,7 @@
         </is>
       </c>
       <c r="I123" t="n">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="J123" t="inlineStr">
         <is>
@@ -6610,7 +6610,7 @@
         </is>
       </c>
       <c r="I124" t="n">
-        <v>68</v>
+        <v>83</v>
       </c>
       <c r="J124" t="inlineStr">
         <is>
@@ -6660,7 +6660,7 @@
         </is>
       </c>
       <c r="I125" t="n">
-        <v>63</v>
+        <v>70</v>
       </c>
       <c r="J125" t="inlineStr">
         <is>
@@ -6710,7 +6710,7 @@
         </is>
       </c>
       <c r="I126" t="n">
-        <v>79</v>
+        <v>69</v>
       </c>
       <c r="J126" t="inlineStr">
         <is>
@@ -6760,7 +6760,7 @@
         </is>
       </c>
       <c r="I127" t="n">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="J127" t="inlineStr">
         <is>
@@ -6810,7 +6810,7 @@
         </is>
       </c>
       <c r="I128" t="n">
-        <v>49</v>
+        <v>32</v>
       </c>
       <c r="J128" t="inlineStr">
         <is>
@@ -6860,7 +6860,7 @@
         </is>
       </c>
       <c r="I129" t="n">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="J129" t="inlineStr">
         <is>
@@ -6910,7 +6910,7 @@
         </is>
       </c>
       <c r="I130" t="n">
-        <v>61</v>
+        <v>74</v>
       </c>
       <c r="J130" t="inlineStr">
         <is>
@@ -6960,7 +6960,7 @@
         </is>
       </c>
       <c r="I131" t="n">
-        <v>77</v>
+        <v>60</v>
       </c>
       <c r="J131" t="inlineStr">
         <is>
@@ -7010,7 +7010,7 @@
         </is>
       </c>
       <c r="I132" t="n">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="J132" t="inlineStr">
         <is>
@@ -7060,7 +7060,7 @@
         </is>
       </c>
       <c r="I133" t="n">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="J133" t="inlineStr">
         <is>
@@ -7110,7 +7110,7 @@
         </is>
       </c>
       <c r="I134" t="n">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="J134" t="inlineStr">
         <is>
@@ -7160,7 +7160,7 @@
         </is>
       </c>
       <c r="I135" t="n">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="J135" t="inlineStr">
         <is>
@@ -7210,7 +7210,7 @@
         </is>
       </c>
       <c r="I136" t="n">
-        <v>39</v>
+        <v>47</v>
       </c>
       <c r="J136" t="inlineStr">
         <is>
@@ -7260,7 +7260,7 @@
         </is>
       </c>
       <c r="I137" t="n">
-        <v>56</v>
+        <v>45</v>
       </c>
       <c r="J137" t="inlineStr">
         <is>
@@ -7310,7 +7310,7 @@
         </is>
       </c>
       <c r="I138" t="n">
-        <v>57</v>
+        <v>63</v>
       </c>
       <c r="J138" t="inlineStr">
         <is>
@@ -7360,7 +7360,7 @@
         </is>
       </c>
       <c r="I139" t="n">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="J139" t="inlineStr">
         <is>
@@ -7410,7 +7410,7 @@
         </is>
       </c>
       <c r="I140" t="n">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="J140" t="inlineStr">
         <is>
@@ -7459,12 +7459,10 @@
           <t>2023-Dec</t>
         </is>
       </c>
-      <c r="I141" t="n">
-        <v>60</v>
-      </c>
+      <c r="I141" t="inlineStr"/>
       <c r="J141" t="inlineStr">
         <is>
-          <t>Sat</t>
+          <t>Absent</t>
         </is>
       </c>
     </row>
@@ -7510,7 +7508,7 @@
         </is>
       </c>
       <c r="I142" t="n">
-        <v>60</v>
+        <v>67</v>
       </c>
       <c r="J142" t="inlineStr">
         <is>
@@ -7560,7 +7558,7 @@
         </is>
       </c>
       <c r="I143" t="n">
-        <v>62</v>
+        <v>51</v>
       </c>
       <c r="J143" t="inlineStr">
         <is>
@@ -7610,7 +7608,7 @@
         </is>
       </c>
       <c r="I144" t="n">
-        <v>31</v>
+        <v>48</v>
       </c>
       <c r="J144" t="inlineStr">
         <is>
@@ -7659,10 +7657,12 @@
           <t>2023-Dec</t>
         </is>
       </c>
-      <c r="I145" t="inlineStr"/>
+      <c r="I145" t="n">
+        <v>48</v>
+      </c>
       <c r="J145" t="inlineStr">
         <is>
-          <t>Absent</t>
+          <t>Sat</t>
         </is>
       </c>
     </row>
@@ -7708,7 +7708,7 @@
         </is>
       </c>
       <c r="I146" t="n">
-        <v>44</v>
+        <v>60</v>
       </c>
       <c r="J146" t="inlineStr">
         <is>
@@ -7758,7 +7758,7 @@
         </is>
       </c>
       <c r="I147" t="n">
-        <v>69</v>
+        <v>56</v>
       </c>
       <c r="J147" t="inlineStr">
         <is>
@@ -7808,7 +7808,7 @@
         </is>
       </c>
       <c r="I148" t="n">
-        <v>55</v>
+        <v>63</v>
       </c>
       <c r="J148" t="inlineStr">
         <is>
@@ -7858,7 +7858,7 @@
         </is>
       </c>
       <c r="I149" t="n">
-        <v>62</v>
+        <v>55</v>
       </c>
       <c r="J149" t="inlineStr">
         <is>
@@ -7908,7 +7908,7 @@
         </is>
       </c>
       <c r="I150" t="n">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="J150" t="inlineStr">
         <is>
@@ -7958,7 +7958,7 @@
         </is>
       </c>
       <c r="I151" t="n">
-        <v>65</v>
+        <v>76</v>
       </c>
       <c r="J151" t="inlineStr">
         <is>
@@ -8008,7 +8008,7 @@
         </is>
       </c>
       <c r="I152" t="n">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="J152" t="inlineStr">
         <is>
@@ -8058,7 +8058,7 @@
         </is>
       </c>
       <c r="I153" t="n">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="J153" t="inlineStr">
         <is>
@@ -8108,7 +8108,7 @@
         </is>
       </c>
       <c r="I154" t="n">
-        <v>57</v>
+        <v>71</v>
       </c>
       <c r="J154" t="inlineStr">
         <is>
@@ -8158,7 +8158,7 @@
         </is>
       </c>
       <c r="I155" t="n">
-        <v>73</v>
+        <v>64</v>
       </c>
       <c r="J155" t="inlineStr">
         <is>
@@ -8208,7 +8208,7 @@
         </is>
       </c>
       <c r="I156" t="n">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="J156" t="inlineStr">
         <is>
@@ -8258,7 +8258,7 @@
         </is>
       </c>
       <c r="I157" t="n">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="J157" t="inlineStr">
         <is>
@@ -8308,7 +8308,7 @@
         </is>
       </c>
       <c r="I158" t="n">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="J158" t="inlineStr">
         <is>
@@ -8358,7 +8358,7 @@
         </is>
       </c>
       <c r="I159" t="n">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="J159" t="inlineStr">
         <is>
@@ -8408,7 +8408,7 @@
         </is>
       </c>
       <c r="I160" t="n">
-        <v>69</v>
+        <v>58</v>
       </c>
       <c r="J160" t="inlineStr">
         <is>
@@ -8458,7 +8458,7 @@
         </is>
       </c>
       <c r="I161" t="n">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="J161" t="inlineStr">
         <is>
@@ -8508,7 +8508,7 @@
         </is>
       </c>
       <c r="I162" t="n">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="J162" t="inlineStr">
         <is>
@@ -8558,7 +8558,7 @@
         </is>
       </c>
       <c r="I163" t="n">
-        <v>75</v>
+        <v>68</v>
       </c>
       <c r="J163" t="inlineStr">
         <is>
@@ -8608,7 +8608,7 @@
         </is>
       </c>
       <c r="I164" t="n">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="J164" t="inlineStr">
         <is>
@@ -8658,7 +8658,7 @@
         </is>
       </c>
       <c r="I165" t="n">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="J165" t="inlineStr">
         <is>
@@ -8708,7 +8708,7 @@
         </is>
       </c>
       <c r="I166" t="n">
-        <v>73</v>
+        <v>60</v>
       </c>
       <c r="J166" t="inlineStr">
         <is>
@@ -8758,7 +8758,7 @@
         </is>
       </c>
       <c r="I167" t="n">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="J167" t="inlineStr">
         <is>
@@ -8808,7 +8808,7 @@
         </is>
       </c>
       <c r="I168" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="J168" t="inlineStr">
         <is>
@@ -8858,7 +8858,7 @@
         </is>
       </c>
       <c r="I169" t="n">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="J169" t="inlineStr">
         <is>
@@ -8908,7 +8908,7 @@
         </is>
       </c>
       <c r="I170" t="n">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="J170" t="inlineStr">
         <is>
@@ -8958,7 +8958,7 @@
         </is>
       </c>
       <c r="I171" t="n">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="J171" t="inlineStr">
         <is>
@@ -9008,7 +9008,7 @@
         </is>
       </c>
       <c r="I172" t="n">
-        <v>58</v>
+        <v>39</v>
       </c>
       <c r="J172" t="inlineStr">
         <is>
@@ -9058,7 +9058,7 @@
         </is>
       </c>
       <c r="I173" t="n">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="J173" t="inlineStr">
         <is>
@@ -9108,7 +9108,7 @@
         </is>
       </c>
       <c r="I174" t="n">
-        <v>66</v>
+        <v>74</v>
       </c>
       <c r="J174" t="inlineStr">
         <is>
@@ -9158,7 +9158,7 @@
         </is>
       </c>
       <c r="I175" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="J175" t="inlineStr">
         <is>
@@ -9208,7 +9208,7 @@
         </is>
       </c>
       <c r="I176" t="n">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="J176" t="inlineStr">
         <is>
@@ -9258,7 +9258,7 @@
         </is>
       </c>
       <c r="I177" t="n">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="J177" t="inlineStr">
         <is>
@@ -9308,7 +9308,7 @@
         </is>
       </c>
       <c r="I178" t="n">
-        <v>56</v>
+        <v>69</v>
       </c>
       <c r="J178" t="inlineStr">
         <is>
@@ -9358,7 +9358,7 @@
         </is>
       </c>
       <c r="I179" t="n">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="J179" t="inlineStr">
         <is>
@@ -9408,7 +9408,7 @@
         </is>
       </c>
       <c r="I180" t="n">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="J180" t="inlineStr">
         <is>
@@ -9458,7 +9458,7 @@
         </is>
       </c>
       <c r="I181" t="n">
-        <v>60</v>
+        <v>67</v>
       </c>
       <c r="J181" t="inlineStr">
         <is>
@@ -9508,7 +9508,7 @@
         </is>
       </c>
       <c r="I182" t="n">
-        <v>62</v>
+        <v>74</v>
       </c>
       <c r="J182" t="inlineStr">
         <is>
@@ -9558,7 +9558,7 @@
         </is>
       </c>
       <c r="I183" t="n">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="J183" t="inlineStr">
         <is>
@@ -9608,7 +9608,7 @@
         </is>
       </c>
       <c r="I184" t="n">
-        <v>66</v>
+        <v>86</v>
       </c>
       <c r="J184" t="inlineStr">
         <is>
@@ -9657,12 +9657,10 @@
           <t>2023-Dec</t>
         </is>
       </c>
-      <c r="I185" t="n">
-        <v>88</v>
-      </c>
+      <c r="I185" t="inlineStr"/>
       <c r="J185" t="inlineStr">
         <is>
-          <t>Sat</t>
+          <t>Absent</t>
         </is>
       </c>
     </row>
@@ -9708,7 +9706,7 @@
         </is>
       </c>
       <c r="I186" t="n">
-        <v>65</v>
+        <v>81</v>
       </c>
       <c r="J186" t="inlineStr">
         <is>
@@ -9758,7 +9756,7 @@
         </is>
       </c>
       <c r="I187" t="n">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="J187" t="inlineStr">
         <is>
@@ -9808,7 +9806,7 @@
         </is>
       </c>
       <c r="I188" t="n">
-        <v>72</v>
+        <v>60</v>
       </c>
       <c r="J188" t="inlineStr">
         <is>
@@ -9858,7 +9856,7 @@
         </is>
       </c>
       <c r="I189" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="J189" t="inlineStr">
         <is>
@@ -9958,7 +9956,7 @@
         </is>
       </c>
       <c r="I191" t="n">
-        <v>58</v>
+        <v>70</v>
       </c>
       <c r="J191" t="inlineStr">
         <is>
@@ -10008,7 +10006,7 @@
         </is>
       </c>
       <c r="I192" t="n">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="J192" t="inlineStr">
         <is>
@@ -10058,7 +10056,7 @@
         </is>
       </c>
       <c r="I193" t="n">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="J193" t="inlineStr">
         <is>
@@ -10107,12 +10105,10 @@
           <t>2023-Dec</t>
         </is>
       </c>
-      <c r="I194" t="n">
-        <v>67</v>
-      </c>
+      <c r="I194" t="inlineStr"/>
       <c r="J194" t="inlineStr">
         <is>
-          <t>Sat</t>
+          <t>Absent</t>
         </is>
       </c>
     </row>
@@ -10158,7 +10154,7 @@
         </is>
       </c>
       <c r="I195" t="n">
-        <v>46</v>
+        <v>68</v>
       </c>
       <c r="J195" t="inlineStr">
         <is>
@@ -10208,7 +10204,7 @@
         </is>
       </c>
       <c r="I196" t="n">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="J196" t="inlineStr">
         <is>
@@ -10258,7 +10254,7 @@
         </is>
       </c>
       <c r="I197" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="J197" t="inlineStr">
         <is>
@@ -10308,7 +10304,7 @@
         </is>
       </c>
       <c r="I198" t="n">
-        <v>53</v>
+        <v>62</v>
       </c>
       <c r="J198" t="inlineStr">
         <is>
@@ -10358,7 +10354,7 @@
         </is>
       </c>
       <c r="I199" t="n">
-        <v>61</v>
+        <v>74</v>
       </c>
       <c r="J199" t="inlineStr">
         <is>
@@ -10408,7 +10404,7 @@
         </is>
       </c>
       <c r="I200" t="n">
-        <v>41</v>
+        <v>52</v>
       </c>
       <c r="J200" t="inlineStr">
         <is>
@@ -10457,10 +10453,12 @@
           <t>2023-Dec</t>
         </is>
       </c>
-      <c r="I201" t="inlineStr"/>
+      <c r="I201" t="n">
+        <v>39</v>
+      </c>
       <c r="J201" t="inlineStr">
         <is>
-          <t>Medical</t>
+          <t>Sat</t>
         </is>
       </c>
     </row>
@@ -10506,7 +10504,7 @@
         </is>
       </c>
       <c r="I202" t="n">
-        <v>79</v>
+        <v>87</v>
       </c>
       <c r="J202" t="inlineStr">
         <is>
@@ -10556,7 +10554,7 @@
         </is>
       </c>
       <c r="I203" t="n">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="J203" t="inlineStr">
         <is>
@@ -10606,7 +10604,7 @@
         </is>
       </c>
       <c r="I204" t="n">
-        <v>65</v>
+        <v>82</v>
       </c>
       <c r="J204" t="inlineStr">
         <is>
@@ -10655,12 +10653,10 @@
           <t>2023-Dec</t>
         </is>
       </c>
-      <c r="I205" t="n">
-        <v>71</v>
-      </c>
+      <c r="I205" t="inlineStr"/>
       <c r="J205" t="inlineStr">
         <is>
-          <t>Sat</t>
+          <t>Medical</t>
         </is>
       </c>
     </row>
@@ -10706,7 +10702,7 @@
         </is>
       </c>
       <c r="I206" t="n">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="J206" t="inlineStr">
         <is>
@@ -10756,7 +10752,7 @@
         </is>
       </c>
       <c r="I207" t="n">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="J207" t="inlineStr">
         <is>
@@ -10806,7 +10802,7 @@
         </is>
       </c>
       <c r="I208" t="n">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="J208" t="inlineStr">
         <is>
@@ -10856,7 +10852,7 @@
         </is>
       </c>
       <c r="I209" t="n">
-        <v>46</v>
+        <v>62</v>
       </c>
       <c r="J209" t="inlineStr">
         <is>
@@ -10906,7 +10902,7 @@
         </is>
       </c>
       <c r="I210" t="n">
-        <v>72</v>
+        <v>80</v>
       </c>
       <c r="J210" t="inlineStr">
         <is>
@@ -10956,7 +10952,7 @@
         </is>
       </c>
       <c r="I211" t="n">
-        <v>72</v>
+        <v>66</v>
       </c>
       <c r="J211" t="inlineStr">
         <is>
@@ -11006,7 +11002,7 @@
         </is>
       </c>
       <c r="I212" t="n">
-        <v>69</v>
+        <v>46</v>
       </c>
       <c r="J212" t="inlineStr">
         <is>
@@ -11056,7 +11052,7 @@
         </is>
       </c>
       <c r="I213" t="n">
-        <v>51</v>
+        <v>68</v>
       </c>
       <c r="J213" t="inlineStr">
         <is>
@@ -11105,10 +11101,12 @@
           <t>2023-Dec</t>
         </is>
       </c>
-      <c r="I214" t="inlineStr"/>
+      <c r="I214" t="n">
+        <v>72</v>
+      </c>
       <c r="J214" t="inlineStr">
         <is>
-          <t>Absent</t>
+          <t>Sat</t>
         </is>
       </c>
     </row>
@@ -11154,7 +11152,7 @@
         </is>
       </c>
       <c r="I215" t="n">
-        <v>64</v>
+        <v>87</v>
       </c>
       <c r="J215" t="inlineStr">
         <is>
@@ -11204,7 +11202,7 @@
         </is>
       </c>
       <c r="I216" t="n">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="J216" t="inlineStr">
         <is>
@@ -11254,7 +11252,7 @@
         </is>
       </c>
       <c r="I217" t="n">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="J217" t="inlineStr">
         <is>
@@ -11353,10 +11351,12 @@
           <t>2023-Dec</t>
         </is>
       </c>
-      <c r="I219" t="inlineStr"/>
+      <c r="I219" t="n">
+        <v>63</v>
+      </c>
       <c r="J219" t="inlineStr">
         <is>
-          <t>Absent</t>
+          <t>Sat</t>
         </is>
       </c>
     </row>
@@ -11402,7 +11402,7 @@
         </is>
       </c>
       <c r="I220" t="n">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="J220" t="inlineStr">
         <is>
@@ -11452,7 +11452,7 @@
         </is>
       </c>
       <c r="I221" t="n">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="J221" t="inlineStr">
         <is>
@@ -11502,7 +11502,7 @@
         </is>
       </c>
       <c r="I222" t="n">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="J222" t="inlineStr">
         <is>
@@ -11552,7 +11552,7 @@
         </is>
       </c>
       <c r="I223" t="n">
-        <v>71</v>
+        <v>58</v>
       </c>
       <c r="J223" t="inlineStr">
         <is>
@@ -11602,7 +11602,7 @@
         </is>
       </c>
       <c r="I224" t="n">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="J224" t="inlineStr">
         <is>
@@ -11652,7 +11652,7 @@
         </is>
       </c>
       <c r="I225" t="n">
-        <v>61</v>
+        <v>74</v>
       </c>
       <c r="J225" t="inlineStr">
         <is>
@@ -11702,7 +11702,7 @@
         </is>
       </c>
       <c r="I226" t="n">
-        <v>55</v>
+        <v>86</v>
       </c>
       <c r="J226" t="inlineStr">
         <is>
@@ -11752,7 +11752,7 @@
         </is>
       </c>
       <c r="I227" t="n">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="J227" t="inlineStr">
         <is>
@@ -11802,7 +11802,7 @@
         </is>
       </c>
       <c r="I228" t="n">
-        <v>64</v>
+        <v>55</v>
       </c>
       <c r="J228" t="inlineStr">
         <is>
@@ -11851,10 +11851,12 @@
           <t>2023-Dec</t>
         </is>
       </c>
-      <c r="I229" t="inlineStr"/>
+      <c r="I229" t="n">
+        <v>70</v>
+      </c>
       <c r="J229" t="inlineStr">
         <is>
-          <t>Absent</t>
+          <t>Sat</t>
         </is>
       </c>
     </row>
@@ -11900,7 +11902,7 @@
         </is>
       </c>
       <c r="I230" t="n">
-        <v>41</v>
+        <v>56</v>
       </c>
       <c r="J230" t="inlineStr">
         <is>
@@ -11950,7 +11952,7 @@
         </is>
       </c>
       <c r="I231" t="n">
-        <v>43</v>
+        <v>59</v>
       </c>
       <c r="J231" t="inlineStr">
         <is>
@@ -12000,7 +12002,7 @@
         </is>
       </c>
       <c r="I232" t="n">
-        <v>62</v>
+        <v>53</v>
       </c>
       <c r="J232" t="inlineStr">
         <is>
@@ -12050,7 +12052,7 @@
         </is>
       </c>
       <c r="I233" t="n">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="J233" t="inlineStr">
         <is>
@@ -12100,7 +12102,7 @@
         </is>
       </c>
       <c r="I234" t="n">
-        <v>78</v>
+        <v>93</v>
       </c>
       <c r="J234" t="inlineStr">
         <is>
@@ -12150,7 +12152,7 @@
         </is>
       </c>
       <c r="I235" t="n">
-        <v>64</v>
+        <v>72</v>
       </c>
       <c r="J235" t="inlineStr">
         <is>
@@ -12200,7 +12202,7 @@
         </is>
       </c>
       <c r="I236" t="n">
-        <v>69</v>
+        <v>55</v>
       </c>
       <c r="J236" t="inlineStr">
         <is>
@@ -12250,7 +12252,7 @@
         </is>
       </c>
       <c r="I237" t="n">
-        <v>50</v>
+        <v>66</v>
       </c>
       <c r="J237" t="inlineStr">
         <is>
@@ -12300,7 +12302,7 @@
         </is>
       </c>
       <c r="I238" t="n">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="J238" t="inlineStr">
         <is>
@@ -12350,7 +12352,7 @@
         </is>
       </c>
       <c r="I239" t="n">
-        <v>65</v>
+        <v>45</v>
       </c>
       <c r="J239" t="inlineStr">
         <is>
@@ -12400,7 +12402,7 @@
         </is>
       </c>
       <c r="I240" t="n">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="J240" t="inlineStr">
         <is>
@@ -12450,7 +12452,7 @@
         </is>
       </c>
       <c r="I241" t="n">
-        <v>60</v>
+        <v>74</v>
       </c>
       <c r="J241" t="inlineStr">
         <is>
@@ -12500,7 +12502,7 @@
         </is>
       </c>
       <c r="I242" t="n">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="J242" t="inlineStr">
         <is>
@@ -12550,7 +12552,7 @@
         </is>
       </c>
       <c r="I243" t="n">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="J243" t="inlineStr">
         <is>
@@ -12600,7 +12602,7 @@
         </is>
       </c>
       <c r="I244" t="n">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="J244" t="inlineStr">
         <is>
@@ -12650,7 +12652,7 @@
         </is>
       </c>
       <c r="I245" t="n">
-        <v>56</v>
+        <v>65</v>
       </c>
       <c r="J245" t="inlineStr">
         <is>
@@ -12700,7 +12702,7 @@
         </is>
       </c>
       <c r="I246" t="n">
-        <v>71</v>
+        <v>61</v>
       </c>
       <c r="J246" t="inlineStr">
         <is>
@@ -12750,7 +12752,7 @@
         </is>
       </c>
       <c r="I247" t="n">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="J247" t="inlineStr">
         <is>
@@ -12799,10 +12801,12 @@
           <t>2023-Dec</t>
         </is>
       </c>
-      <c r="I248" t="inlineStr"/>
+      <c r="I248" t="n">
+        <v>80</v>
+      </c>
       <c r="J248" t="inlineStr">
         <is>
-          <t>Absent</t>
+          <t>Sat</t>
         </is>
       </c>
     </row>
@@ -12848,7 +12852,7 @@
         </is>
       </c>
       <c r="I249" t="n">
-        <v>60</v>
+        <v>67</v>
       </c>
       <c r="J249" t="inlineStr">
         <is>
@@ -12898,7 +12902,7 @@
         </is>
       </c>
       <c r="I250" t="n">
-        <v>69</v>
+        <v>58</v>
       </c>
       <c r="J250" t="inlineStr">
         <is>
@@ -12948,7 +12952,7 @@
         </is>
       </c>
       <c r="I251" t="n">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="J251" t="inlineStr">
         <is>
@@ -12998,7 +13002,7 @@
         </is>
       </c>
       <c r="I252" t="n">
-        <v>54</v>
+        <v>40</v>
       </c>
       <c r="J252" t="inlineStr">
         <is>
@@ -13048,7 +13052,7 @@
         </is>
       </c>
       <c r="I253" t="n">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="J253" t="inlineStr">
         <is>
@@ -13098,7 +13102,7 @@
         </is>
       </c>
       <c r="I254" t="n">
-        <v>78</v>
+        <v>59</v>
       </c>
       <c r="J254" t="inlineStr">
         <is>
@@ -13148,7 +13152,7 @@
         </is>
       </c>
       <c r="I255" t="n">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="J255" t="inlineStr">
         <is>
@@ -13198,7 +13202,7 @@
         </is>
       </c>
       <c r="I256" t="n">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="J256" t="inlineStr">
         <is>
@@ -13248,7 +13252,7 @@
         </is>
       </c>
       <c r="I257" t="n">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="J257" t="inlineStr">
         <is>
@@ -13298,7 +13302,7 @@
         </is>
       </c>
       <c r="I258" t="n">
-        <v>73</v>
+        <v>82</v>
       </c>
       <c r="J258" t="inlineStr">
         <is>
@@ -13348,7 +13352,7 @@
         </is>
       </c>
       <c r="I259" t="n">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="J259" t="inlineStr">
         <is>
@@ -13398,7 +13402,7 @@
         </is>
       </c>
       <c r="I260" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="J260" t="inlineStr">
         <is>
@@ -13448,7 +13452,7 @@
         </is>
       </c>
       <c r="I261" t="n">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="J261" t="inlineStr">
         <is>
@@ -13498,7 +13502,7 @@
         </is>
       </c>
       <c r="I262" t="n">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="J262" t="inlineStr">
         <is>
@@ -13548,7 +13552,7 @@
         </is>
       </c>
       <c r="I263" t="n">
-        <v>38</v>
+        <v>49</v>
       </c>
       <c r="J263" t="inlineStr">
         <is>
@@ -13648,7 +13652,7 @@
         </is>
       </c>
       <c r="I265" t="n">
-        <v>78</v>
+        <v>66</v>
       </c>
       <c r="J265" t="inlineStr">
         <is>
@@ -13698,7 +13702,7 @@
         </is>
       </c>
       <c r="I266" t="n">
-        <v>44</v>
+        <v>55</v>
       </c>
       <c r="J266" t="inlineStr">
         <is>
@@ -13748,7 +13752,7 @@
         </is>
       </c>
       <c r="I267" t="n">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="J267" t="inlineStr">
         <is>
@@ -13797,10 +13801,12 @@
           <t>2023-Dec</t>
         </is>
       </c>
-      <c r="I268" t="inlineStr"/>
+      <c r="I268" t="n">
+        <v>77</v>
+      </c>
       <c r="J268" t="inlineStr">
         <is>
-          <t>Absent</t>
+          <t>Sat</t>
         </is>
       </c>
     </row>
@@ -13846,7 +13852,7 @@
         </is>
       </c>
       <c r="I269" t="n">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="J269" t="inlineStr">
         <is>
@@ -13896,7 +13902,7 @@
         </is>
       </c>
       <c r="I270" t="n">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="J270" t="inlineStr">
         <is>
@@ -13945,10 +13951,12 @@
           <t>2023-Dec</t>
         </is>
       </c>
-      <c r="I271" t="inlineStr"/>
+      <c r="I271" t="n">
+        <v>84</v>
+      </c>
       <c r="J271" t="inlineStr">
         <is>
-          <t>Medical</t>
+          <t>Sat</t>
         </is>
       </c>
     </row>
@@ -13993,10 +14001,12 @@
           <t>2023-Dec</t>
         </is>
       </c>
-      <c r="I272" t="inlineStr"/>
+      <c r="I272" t="n">
+        <v>52</v>
+      </c>
       <c r="J272" t="inlineStr">
         <is>
-          <t>Absent</t>
+          <t>Sat</t>
         </is>
       </c>
     </row>
@@ -14042,7 +14052,7 @@
         </is>
       </c>
       <c r="I273" t="n">
-        <v>60</v>
+        <v>52</v>
       </c>
       <c r="J273" t="inlineStr">
         <is>
@@ -14092,7 +14102,7 @@
         </is>
       </c>
       <c r="I274" t="n">
-        <v>54</v>
+        <v>63</v>
       </c>
       <c r="J274" t="inlineStr">
         <is>
@@ -14142,7 +14152,7 @@
         </is>
       </c>
       <c r="I275" t="n">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="J275" t="inlineStr">
         <is>
@@ -14192,7 +14202,7 @@
         </is>
       </c>
       <c r="I276" t="n">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="J276" t="inlineStr">
         <is>
@@ -14242,7 +14252,7 @@
         </is>
       </c>
       <c r="I277" t="n">
-        <v>82</v>
+        <v>70</v>
       </c>
       <c r="J277" t="inlineStr">
         <is>
@@ -14292,7 +14302,7 @@
         </is>
       </c>
       <c r="I278" t="n">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="J278" t="inlineStr">
         <is>
@@ -14341,12 +14351,10 @@
           <t>2023-Dec</t>
         </is>
       </c>
-      <c r="I279" t="n">
-        <v>65</v>
-      </c>
+      <c r="I279" t="inlineStr"/>
       <c r="J279" t="inlineStr">
         <is>
-          <t>Sat</t>
+          <t>Absent</t>
         </is>
       </c>
     </row>
@@ -14392,7 +14400,7 @@
         </is>
       </c>
       <c r="I280" t="n">
-        <v>73</v>
+        <v>57</v>
       </c>
       <c r="J280" t="inlineStr">
         <is>
@@ -14442,7 +14450,7 @@
         </is>
       </c>
       <c r="I281" t="n">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="J281" t="inlineStr">
         <is>
@@ -14492,7 +14500,7 @@
         </is>
       </c>
       <c r="I282" t="n">
-        <v>59</v>
+        <v>69</v>
       </c>
       <c r="J282" t="inlineStr">
         <is>
@@ -14542,7 +14550,7 @@
         </is>
       </c>
       <c r="I283" t="n">
-        <v>65</v>
+        <v>55</v>
       </c>
       <c r="J283" t="inlineStr">
         <is>
@@ -14592,7 +14600,7 @@
         </is>
       </c>
       <c r="I284" t="n">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="J284" t="inlineStr">
         <is>
@@ -14642,7 +14650,7 @@
         </is>
       </c>
       <c r="I285" t="n">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="J285" t="inlineStr">
         <is>
@@ -14692,7 +14700,7 @@
         </is>
       </c>
       <c r="I286" t="n">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="J286" t="inlineStr">
         <is>
@@ -14741,12 +14749,10 @@
           <t>2023-Dec</t>
         </is>
       </c>
-      <c r="I287" t="n">
-        <v>40</v>
-      </c>
+      <c r="I287" t="inlineStr"/>
       <c r="J287" t="inlineStr">
         <is>
-          <t>Sat</t>
+          <t>Absent</t>
         </is>
       </c>
     </row>
@@ -14792,7 +14798,7 @@
         </is>
       </c>
       <c r="I288" t="n">
-        <v>57</v>
+        <v>70</v>
       </c>
       <c r="J288" t="inlineStr">
         <is>
@@ -14842,7 +14848,7 @@
         </is>
       </c>
       <c r="I289" t="n">
-        <v>66</v>
+        <v>42</v>
       </c>
       <c r="J289" t="inlineStr">
         <is>
@@ -14892,7 +14898,7 @@
         </is>
       </c>
       <c r="I290" t="n">
-        <v>66</v>
+        <v>54</v>
       </c>
       <c r="J290" t="inlineStr">
         <is>
@@ -14942,7 +14948,7 @@
         </is>
       </c>
       <c r="I291" t="n">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="J291" t="inlineStr">
         <is>
@@ -14992,7 +14998,7 @@
         </is>
       </c>
       <c r="I292" t="n">
-        <v>80</v>
+        <v>62</v>
       </c>
       <c r="J292" t="inlineStr">
         <is>
@@ -15042,7 +15048,7 @@
         </is>
       </c>
       <c r="I293" t="n">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="J293" t="inlineStr">
         <is>
@@ -15092,7 +15098,7 @@
         </is>
       </c>
       <c r="I294" t="n">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="J294" t="inlineStr">
         <is>
@@ -15142,7 +15148,7 @@
         </is>
       </c>
       <c r="I295" t="n">
-        <v>59</v>
+        <v>52</v>
       </c>
       <c r="J295" t="inlineStr">
         <is>
@@ -15192,7 +15198,7 @@
         </is>
       </c>
       <c r="I296" t="n">
-        <v>51</v>
+        <v>44</v>
       </c>
       <c r="J296" t="inlineStr">
         <is>
@@ -15242,7 +15248,7 @@
         </is>
       </c>
       <c r="I297" t="n">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="J297" t="inlineStr">
         <is>
@@ -15292,7 +15298,7 @@
         </is>
       </c>
       <c r="I298" t="n">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="J298" t="inlineStr">
         <is>
@@ -15342,7 +15348,7 @@
         </is>
       </c>
       <c r="I299" t="n">
-        <v>74</v>
+        <v>83</v>
       </c>
       <c r="J299" t="inlineStr">
         <is>
@@ -15392,7 +15398,7 @@
         </is>
       </c>
       <c r="I300" t="n">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="J300" t="inlineStr">
         <is>
@@ -15442,7 +15448,7 @@
         </is>
       </c>
       <c r="I301" t="n">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="J301" t="inlineStr">
         <is>
@@ -15492,7 +15498,7 @@
         </is>
       </c>
       <c r="I302" t="n">
-        <v>59</v>
+        <v>74</v>
       </c>
       <c r="J302" t="inlineStr">
         <is>
@@ -15592,7 +15598,7 @@
         </is>
       </c>
       <c r="I304" t="n">
-        <v>61</v>
+        <v>71</v>
       </c>
       <c r="J304" t="inlineStr">
         <is>
@@ -15642,7 +15648,7 @@
         </is>
       </c>
       <c r="I305" t="n">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="J305" t="inlineStr">
         <is>
@@ -15692,7 +15698,7 @@
         </is>
       </c>
       <c r="I306" t="n">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="J306" t="inlineStr">
         <is>
@@ -15742,7 +15748,7 @@
         </is>
       </c>
       <c r="I307" t="n">
-        <v>84</v>
+        <v>65</v>
       </c>
       <c r="J307" t="inlineStr">
         <is>
@@ -15792,7 +15798,7 @@
         </is>
       </c>
       <c r="I308" t="n">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="J308" t="inlineStr">
         <is>
@@ -15841,12 +15847,10 @@
           <t>2023-Dec</t>
         </is>
       </c>
-      <c r="I309" t="n">
-        <v>62</v>
-      </c>
+      <c r="I309" t="inlineStr"/>
       <c r="J309" t="inlineStr">
         <is>
-          <t>Sat</t>
+          <t>Absent</t>
         </is>
       </c>
     </row>
@@ -15892,7 +15896,7 @@
         </is>
       </c>
       <c r="I310" t="n">
-        <v>79</v>
+        <v>69</v>
       </c>
       <c r="J310" t="inlineStr">
         <is>
@@ -15942,7 +15946,7 @@
         </is>
       </c>
       <c r="I311" t="n">
-        <v>69</v>
+        <v>53</v>
       </c>
       <c r="J311" t="inlineStr">
         <is>
@@ -15992,7 +15996,7 @@
         </is>
       </c>
       <c r="I312" t="n">
-        <v>80</v>
+        <v>68</v>
       </c>
       <c r="J312" t="inlineStr">
         <is>
@@ -16042,7 +16046,7 @@
         </is>
       </c>
       <c r="I313" t="n">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="J313" t="inlineStr">
         <is>
@@ -16092,7 +16096,7 @@
         </is>
       </c>
       <c r="I314" t="n">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="J314" t="inlineStr">
         <is>
@@ -16142,7 +16146,7 @@
         </is>
       </c>
       <c r="I315" t="n">
-        <v>70</v>
+        <v>77</v>
       </c>
       <c r="J315" t="inlineStr">
         <is>
@@ -16192,7 +16196,7 @@
         </is>
       </c>
       <c r="I316" t="n">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="J316" t="inlineStr">
         <is>
@@ -16242,7 +16246,7 @@
         </is>
       </c>
       <c r="I317" t="n">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="J317" t="inlineStr">
         <is>
@@ -16291,10 +16295,12 @@
           <t>2023-Dec</t>
         </is>
       </c>
-      <c r="I318" t="inlineStr"/>
+      <c r="I318" t="n">
+        <v>62</v>
+      </c>
       <c r="J318" t="inlineStr">
         <is>
-          <t>Absent</t>
+          <t>Sat</t>
         </is>
       </c>
     </row>
@@ -16340,7 +16346,7 @@
         </is>
       </c>
       <c r="I319" t="n">
-        <v>46</v>
+        <v>58</v>
       </c>
       <c r="J319" t="inlineStr">
         <is>
@@ -16390,7 +16396,7 @@
         </is>
       </c>
       <c r="I320" t="n">
-        <v>63</v>
+        <v>54</v>
       </c>
       <c r="J320" t="inlineStr">
         <is>
@@ -16439,10 +16445,12 @@
           <t>2023-Dec</t>
         </is>
       </c>
-      <c r="I321" t="inlineStr"/>
+      <c r="I321" t="n">
+        <v>68</v>
+      </c>
       <c r="J321" t="inlineStr">
         <is>
-          <t>Absent</t>
+          <t>Sat</t>
         </is>
       </c>
     </row>
@@ -16488,7 +16496,7 @@
         </is>
       </c>
       <c r="I322" t="n">
-        <v>66</v>
+        <v>41</v>
       </c>
       <c r="J322" t="inlineStr">
         <is>
@@ -16538,7 +16546,7 @@
         </is>
       </c>
       <c r="I323" t="n">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="J323" t="inlineStr">
         <is>
@@ -16588,7 +16596,7 @@
         </is>
       </c>
       <c r="I324" t="n">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="J324" t="inlineStr">
         <is>
@@ -16638,7 +16646,7 @@
         </is>
       </c>
       <c r="I325" t="n">
-        <v>53</v>
+        <v>60</v>
       </c>
       <c r="J325" t="inlineStr">
         <is>
@@ -16688,7 +16696,7 @@
         </is>
       </c>
       <c r="I326" t="n">
-        <v>59</v>
+        <v>70</v>
       </c>
       <c r="J326" t="inlineStr">
         <is>
@@ -16738,7 +16746,7 @@
         </is>
       </c>
       <c r="I327" t="n">
-        <v>53</v>
+        <v>71</v>
       </c>
       <c r="J327" t="inlineStr">
         <is>
@@ -16788,7 +16796,7 @@
         </is>
       </c>
       <c r="I328" t="n">
-        <v>54</v>
+        <v>65</v>
       </c>
       <c r="J328" t="inlineStr">
         <is>
@@ -16838,7 +16846,7 @@
         </is>
       </c>
       <c r="I329" t="n">
-        <v>54</v>
+        <v>47</v>
       </c>
       <c r="J329" t="inlineStr">
         <is>
@@ -16888,7 +16896,7 @@
         </is>
       </c>
       <c r="I330" t="n">
-        <v>50</v>
+        <v>64</v>
       </c>
       <c r="J330" t="inlineStr">
         <is>
@@ -16938,7 +16946,7 @@
         </is>
       </c>
       <c r="I331" t="n">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="J331" t="inlineStr">
         <is>
@@ -16988,7 +16996,7 @@
         </is>
       </c>
       <c r="I332" t="n">
-        <v>73</v>
+        <v>66</v>
       </c>
       <c r="J332" t="inlineStr">
         <is>
@@ -17038,7 +17046,7 @@
         </is>
       </c>
       <c r="I333" t="n">
-        <v>64</v>
+        <v>78</v>
       </c>
       <c r="J333" t="inlineStr">
         <is>
@@ -17088,7 +17096,7 @@
         </is>
       </c>
       <c r="I334" t="n">
-        <v>39</v>
+        <v>53</v>
       </c>
       <c r="J334" t="inlineStr">
         <is>
@@ -17138,7 +17146,7 @@
         </is>
       </c>
       <c r="I335" t="n">
-        <v>35</v>
+        <v>50</v>
       </c>
       <c r="J335" t="inlineStr">
         <is>
@@ -17188,7 +17196,7 @@
         </is>
       </c>
       <c r="I336" t="n">
-        <v>71</v>
+        <v>79</v>
       </c>
       <c r="J336" t="inlineStr">
         <is>
@@ -17238,7 +17246,7 @@
         </is>
       </c>
       <c r="I337" t="n">
-        <v>71</v>
+        <v>61</v>
       </c>
       <c r="J337" t="inlineStr">
         <is>
@@ -17288,7 +17296,7 @@
         </is>
       </c>
       <c r="I338" t="n">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="J338" t="inlineStr">
         <is>
@@ -17338,7 +17346,7 @@
         </is>
       </c>
       <c r="I339" t="n">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="J339" t="inlineStr">
         <is>
@@ -17388,7 +17396,7 @@
         </is>
       </c>
       <c r="I340" t="n">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="J340" t="inlineStr">
         <is>
@@ -17438,7 +17446,7 @@
         </is>
       </c>
       <c r="I341" t="n">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="J341" t="inlineStr">
         <is>
@@ -17488,7 +17496,7 @@
         </is>
       </c>
       <c r="I342" t="n">
-        <v>57</v>
+        <v>47</v>
       </c>
       <c r="J342" t="inlineStr">
         <is>
@@ -17537,10 +17545,12 @@
           <t>2023-Dec</t>
         </is>
       </c>
-      <c r="I343" t="inlineStr"/>
+      <c r="I343" t="n">
+        <v>46</v>
+      </c>
       <c r="J343" t="inlineStr">
         <is>
-          <t>Absent</t>
+          <t>Sat</t>
         </is>
       </c>
     </row>
@@ -17586,7 +17596,7 @@
         </is>
       </c>
       <c r="I344" t="n">
-        <v>72</v>
+        <v>62</v>
       </c>
       <c r="J344" t="inlineStr">
         <is>
@@ -17636,7 +17646,7 @@
         </is>
       </c>
       <c r="I345" t="n">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="J345" t="inlineStr">
         <is>
@@ -17686,7 +17696,7 @@
         </is>
       </c>
       <c r="I346" t="n">
-        <v>72</v>
+        <v>79</v>
       </c>
       <c r="J346" t="inlineStr">
         <is>
@@ -17736,7 +17746,7 @@
         </is>
       </c>
       <c r="I347" t="n">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="J347" t="inlineStr">
         <is>
@@ -17786,7 +17796,7 @@
         </is>
       </c>
       <c r="I348" t="n">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="J348" t="inlineStr">
         <is>
@@ -17836,7 +17846,7 @@
         </is>
       </c>
       <c r="I349" t="n">
-        <v>70</v>
+        <v>56</v>
       </c>
       <c r="J349" t="inlineStr">
         <is>
@@ -17936,7 +17946,7 @@
         </is>
       </c>
       <c r="I351" t="n">
-        <v>62</v>
+        <v>53</v>
       </c>
       <c r="J351" t="inlineStr">
         <is>
@@ -17986,7 +17996,7 @@
         </is>
       </c>
       <c r="I352" t="n">
-        <v>57</v>
+        <v>63</v>
       </c>
       <c r="J352" t="inlineStr">
         <is>
@@ -18036,7 +18046,7 @@
         </is>
       </c>
       <c r="I353" t="n">
-        <v>44</v>
+        <v>64</v>
       </c>
       <c r="J353" t="inlineStr">
         <is>
@@ -18136,7 +18146,7 @@
         </is>
       </c>
       <c r="I355" t="n">
-        <v>55</v>
+        <v>68</v>
       </c>
       <c r="J355" t="inlineStr">
         <is>
@@ -18186,7 +18196,7 @@
         </is>
       </c>
       <c r="I356" t="n">
-        <v>64</v>
+        <v>55</v>
       </c>
       <c r="J356" t="inlineStr">
         <is>
@@ -18236,7 +18246,7 @@
         </is>
       </c>
       <c r="I357" t="n">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="J357" t="inlineStr">
         <is>
@@ -18336,7 +18346,7 @@
         </is>
       </c>
       <c r="I359" t="n">
-        <v>42</v>
+        <v>53</v>
       </c>
       <c r="J359" t="inlineStr">
         <is>
@@ -18386,7 +18396,7 @@
         </is>
       </c>
       <c r="I360" t="n">
-        <v>47</v>
+        <v>56</v>
       </c>
       <c r="J360" t="inlineStr">
         <is>
@@ -18436,7 +18446,7 @@
         </is>
       </c>
       <c r="I361" t="n">
-        <v>42</v>
+        <v>73</v>
       </c>
       <c r="J361" t="inlineStr">
         <is>
@@ -18486,7 +18496,7 @@
         </is>
       </c>
       <c r="I362" t="n">
-        <v>61</v>
+        <v>52</v>
       </c>
       <c r="J362" t="inlineStr">
         <is>
@@ -18536,7 +18546,7 @@
         </is>
       </c>
       <c r="I363" t="n">
-        <v>67</v>
+        <v>54</v>
       </c>
       <c r="J363" t="inlineStr">
         <is>

</xml_diff>